<commit_message>
Conversion Prompt Changes and Utility Conversions
CONVERSION_GUIDE Iteration through files:
 FindRoot, HalfUpFormat, UtilException, AdaptiveRangeKutta.
</commit_message>
<xml_diff>
--- a/tools/reports/Utility.xlsx
+++ b/tools/reports/Utility.xlsx
@@ -615,22 +615,22 @@
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.039742</v>
+        <v>0.017579</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -639,7 +639,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" t="b">
         <v>0</v>
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -850,7 +850,7 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -936,25 +936,25 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.3333</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N5" t="n">
-        <v>0.021482</v>
+        <v>0.019196</v>
       </c>
       <c r="O5" t="n">
         <v>0</v>
@@ -963,10 +963,10 @@
         <v>0</v>
       </c>
       <c r="Q5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -1058,7 +1058,7 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O6" t="n">
         <v>0</v>
@@ -1148,25 +1148,25 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N7" t="n">
-        <v>0.021482</v>
+        <v>0.015831</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
@@ -1175,10 +1175,10 @@
         <v>0</v>
       </c>
       <c r="Q7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>1</v>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O8" t="n">
         <v>0</v>
@@ -1382,7 +1382,7 @@
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O9" t="n">
         <v>0</v>
@@ -1494,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1584,25 +1584,25 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N11" t="n">
-        <v>0.021482</v>
+        <v>0.032367</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
@@ -1611,10 +1611,10 @@
         <v>0</v>
       </c>
       <c r="Q11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>3</v>
@@ -1688,13 +1688,13 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.021482</v>
+        <v>0.101819</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -1718,7 +1718,7 @@
         <v>1</v>
       </c>
       <c r="R12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
@@ -1796,13 +1796,13 @@
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -1814,7 +1814,7 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0.021482</v>
+        <v>0.07298499999999999</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
@@ -1826,7 +1826,7 @@
         <v>1</v>
       </c>
       <c r="R13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>4</v>
@@ -1918,7 +1918,7 @@
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -2011,22 +2011,22 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
@@ -2035,10 +2035,10 @@
         <v>0</v>
       </c>
       <c r="Q15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
         <v>5</v>
@@ -2130,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O16" t="n">
         <v>0</v>
@@ -2238,7 +2238,7 @@
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
@@ -2331,22 +2331,22 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K18" t="n">
         <v>1</v>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N18" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O18" t="n">
         <v>0</v>
@@ -2454,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O19" t="n">
         <v>0</v>
@@ -2540,13 +2540,13 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0.021482</v>
+        <v>0.017579</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
@@ -2570,7 +2570,7 @@
         <v>1</v>
       </c>
       <c r="R20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S20" t="n">
         <v>0</v>
@@ -2644,34 +2644,34 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N21" t="n">
-        <v>0.039742</v>
+        <v>0.019196</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>0.001107</v>
       </c>
       <c r="P21" t="b">
         <v>0</v>
       </c>
       <c r="Q21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R21" t="b">
         <v>0</v>
@@ -2752,25 +2752,25 @@
       </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K22" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M22" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="N22" t="n">
-        <v>0.021482</v>
+        <v>0.014958</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
@@ -2859,22 +2859,22 @@
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N23" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -2883,10 +2883,10 @@
         <v>0</v>
       </c>
       <c r="Q23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
         <v>14</v>
@@ -2963,31 +2963,31 @@
         <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>0.6667</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N24" t="n">
-        <v>0.039742</v>
+        <v>0.022822</v>
       </c>
       <c r="O24" t="n">
-        <v>0</v>
+        <v>0.003322</v>
       </c>
       <c r="P24" t="b">
         <v>0</v>
       </c>
       <c r="Q24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R24" t="b">
         <v>0</v>
@@ -3080,13 +3080,13 @@
         <v>1</v>
       </c>
       <c r="L25" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N25" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
@@ -3175,22 +3175,22 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M26" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="N26" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
@@ -3199,10 +3199,10 @@
         <v>0</v>
       </c>
       <c r="Q26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S26" t="n">
         <v>1</v>
@@ -3276,37 +3276,37 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27" t="n">
-        <v>0.021482</v>
+        <v>0.105277</v>
       </c>
       <c r="O27" t="n">
-        <v>0</v>
+        <v>0.009967</v>
       </c>
       <c r="P27" t="b">
         <v>0</v>
       </c>
       <c r="Q27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>5</v>
@@ -3383,22 +3383,22 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N28" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
@@ -3407,10 +3407,10 @@
         <v>0</v>
       </c>
       <c r="Q28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S28" t="n">
         <v>1</v>
@@ -3487,22 +3487,22 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M29" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N29" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
@@ -3511,10 +3511,10 @@
         <v>0</v>
       </c>
       <c r="Q29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S29" t="n">
         <v>4</v>
@@ -3606,7 +3606,7 @@
         <v>0</v>
       </c>
       <c r="N30" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O30" t="n">
         <v>0</v>
@@ -3695,22 +3695,22 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N31" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O31" t="n">
         <v>0</v>
@@ -3719,10 +3719,10 @@
         <v>0</v>
       </c>
       <c r="Q31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R31" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S31" t="n">
         <v>4</v>
@@ -3814,7 +3814,7 @@
         <v>0</v>
       </c>
       <c r="N32" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O32" t="n">
         <v>0</v>
@@ -3903,22 +3903,22 @@
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N33" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O33" t="n">
         <v>0</v>
@@ -3927,10 +3927,10 @@
         <v>0</v>
       </c>
       <c r="Q33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S33" t="n">
         <v>1</v>
@@ -4026,7 +4026,7 @@
         <v>0</v>
       </c>
       <c r="N34" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O34" t="n">
         <v>0</v>
@@ -4119,22 +4119,22 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N35" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O35" t="n">
         <v>0</v>
@@ -4143,10 +4143,10 @@
         <v>0</v>
       </c>
       <c r="Q35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S35" t="n">
         <v>1</v>
@@ -4220,37 +4220,37 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>0.3333</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N36" t="n">
-        <v>0.021482</v>
+        <v>0.020201</v>
       </c>
       <c r="O36" t="n">
-        <v>0</v>
+        <v>0.000554</v>
       </c>
       <c r="P36" t="b">
         <v>0</v>
       </c>
       <c r="Q36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S36" t="n">
         <v>2</v>
@@ -4346,7 +4346,7 @@
         <v>0</v>
       </c>
       <c r="N37" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O37" t="n">
         <v>0</v>
@@ -4435,22 +4435,22 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N38" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O38" t="n">
         <v>0</v>
@@ -4459,10 +4459,10 @@
         <v>0</v>
       </c>
       <c r="Q38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S38" t="n">
         <v>2</v>
@@ -4554,7 +4554,7 @@
         <v>0</v>
       </c>
       <c r="N39" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
@@ -4658,7 +4658,7 @@
         <v>0</v>
       </c>
       <c r="N40" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O40" t="n">
         <v>0</v>
@@ -4747,22 +4747,22 @@
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N41" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
@@ -4771,10 +4771,10 @@
         <v>0</v>
       </c>
       <c r="Q41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S41" t="n">
         <v>3</v>
@@ -4851,22 +4851,22 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N42" t="n">
-        <v>0.021482</v>
+        <v>0.012336</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
@@ -4875,10 +4875,10 @@
         <v>0</v>
       </c>
       <c r="Q42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S42" t="n">
         <v>0</v>
@@ -4960,37 +4960,37 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>0.3077</v>
       </c>
       <c r="L43" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N43" t="n">
-        <v>0.021482</v>
+        <v>0.094266</v>
       </c>
       <c r="O43" t="n">
-        <v>0</v>
+        <v>0.023256</v>
       </c>
       <c r="P43" t="b">
         <v>0</v>
       </c>
       <c r="Q43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R43" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S43" t="n">
         <v>14</v>
@@ -5068,25 +5068,25 @@
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M44" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N44" t="n">
-        <v>0.021482</v>
+        <v>0.015831</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
@@ -5095,10 +5095,10 @@
         <v>0</v>
       </c>
       <c r="Q44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S44" t="n">
         <v>2</v>
@@ -5176,13 +5176,13 @@
       </c>
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K45" t="n">
         <v>0</v>
@@ -5194,7 +5194,7 @@
         <v>0</v>
       </c>
       <c r="N45" t="n">
-        <v>0.021482</v>
+        <v>0.07234500000000001</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
@@ -5206,7 +5206,7 @@
         <v>1</v>
       </c>
       <c r="R45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S45" t="n">
         <v>0</v>
@@ -5262,7 +5262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G235"/>
+  <dimension ref="A1:G274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13490,6 +13490,1371 @@
       </c>
       <c r="G235" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>AdaptiveRungeKutta</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>AdaptiveRungeKutta.java</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UtilException</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>UtilException</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G236" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Constraint</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Constraint.java</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G237" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>DescriptiveStatistics</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>DescriptiveStatistics.java</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G238" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>ExponentFormat</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>ExponentFormat.java</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G239" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>HTMLFormat</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>HTMLFormat.java</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G240" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Integrator</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Integrator.java</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UtilException</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>UtilException</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G241" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardt2</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardt2.java</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G242" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardt2</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardt2.java</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G243" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtConstrained</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtConstrained.java</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Constraint</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Constraint</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G244" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtConstrained</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtConstrained.java</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G245" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized.java</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.LevenbergMarquardt2</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardt2</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G246" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized.java</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.LevenbergMarquardtConstrained</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtConstrained</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G247" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized.java</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Constraint</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Constraint</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G248" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>LevenbergMarquardtParameterized.java</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G249" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>LinearLeastSquares</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>LinearLeastSquares.java</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G250" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>LinearLeastSquares</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>LinearLeastSquares.java</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G251" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>LinearRegression</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>LinearRegression.java</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.LazyEvaluate</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>LazyEvaluate</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G252" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>LinearRegression</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>LinearRegression.java</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G253" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Math2.java</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.FindRoot</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>FindRoot</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G254" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>MCIntegrator</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>MCIntegrator.java</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G255" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine.java</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValueMC</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>UncertainValueMC</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G256" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine.java</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G257" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>MCUncertaintyEngine.java</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.DescriptiveStatistics</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>DescriptiveStatistics</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G258" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>MultiDHistogram</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>MultiDHistogram.java</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G259" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>PoissonDeviate</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>PoissonDeviate.java</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G260" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>ProgressEvent</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>ProgressEvent.java</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G261" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Simplex</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Simplex.java</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UtilException</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>UtilException</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G262" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>StageRelocation</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>StageRelocation.java</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G263" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>StageRelocation</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>StageRelocation.java</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Simplex</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Simplex</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G264" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Translate2D</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Translate2D.java</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G265" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Translate2D</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Translate2D.java</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Simplex</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Simplex</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G266" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Translate2D</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Translate2D.java</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UtilException</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>UtilException</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G267" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Translate2D</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Translate2D.java</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G268" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>UncertainValue</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>UncertainValue.java</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G269" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>UncertainValue2.java</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.ExponentFormat</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>ExponentFormat</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G270" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>UncertainValue2.java</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>HalfUpFormat</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G271" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>UncertainValue2.java</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UtilException</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>UtilException</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G272" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>UncertainValue2.java</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.Math2</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Math2</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G273" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>UncertainValueMC</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>UncertainValueMC.java</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>gov.nist.microanalysis.Utility.UncertainValue2</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>UncertainValue2</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="G274" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -13528,7 +14893,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -13541,557 +14906,557 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Integrator</t>
+          <t>Constraint</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LevenbergMarquardt2</t>
+          <t>DescriptiveStatistics</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtConstrained</t>
+          <t>ExponentFormat</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LinearLeastSquares</t>
+          <t>FindRoot</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LinearLeastSquaresMS</t>
+          <t>HTMLFormat</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AutoComplete</t>
+          <t>HalfUpFormat</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ComboBoxCellEditor</t>
+          <t>Integrator</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Constraint</t>
+          <t>LazyEvaluate</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>CSVReader</t>
+          <t>LevenbergMarquardt2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DescriptiveStatistics</t>
+          <t>LevenbergMarquardtConstrained</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>EachRowEditor</t>
+          <t>LevenbergMarquardtParameterized</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ElementComboBoxModel</t>
+          <t>LinearLeastSquares</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ElementTreePanel</t>
+          <t>LinearLeastSquaresMS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ExponentFormat</t>
+          <t>LinearRegression</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FindRoot</t>
+          <t>MCIntegrator</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>HalfUpFormat</t>
+          <t>MCUncertaintyEngine</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Histogram</t>
+          <t>Math2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>HTMLFormat</t>
+          <t>MultiDHistogram</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>HTMLList</t>
+          <t>PoissonDeviate</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>HtmlSelection</t>
+          <t>ProgressEvent</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Interval</t>
+          <t>Simplex</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LazyEvaluate</t>
+          <t>StageRelocation</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtParameterized</t>
+          <t>Translate2D</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LinearRegression</t>
+          <t>UncertainValue</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Math2</t>
+          <t>UncertainValue2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MCIntegrator</t>
+          <t>UncertainValueMC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MCUncertaintyEngine</t>
+          <t>UtilException</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B30" t="n">
         <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MemberSet</t>
+          <t>AutoComplete</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>27</v>
+        <v>3</v>
       </c>
       <c r="B31" t="n">
         <v>1</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MultiDHistogram</t>
+          <t>ComboBoxCellEditor</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="B32" t="n">
         <v>1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pair</t>
+          <t>CSVReader</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="B33" t="n">
         <v>1</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PoissonDeviate</t>
+          <t>EachRowEditor</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="B34" t="n">
         <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PrintUtilities</t>
+          <t>ElementComboBoxModel</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="B35" t="n">
         <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ProgressEvent</t>
+          <t>ElementTreePanel</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="B36" t="n">
         <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Simplex</t>
+          <t>Histogram</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="B37" t="n">
         <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SpectrumPropertiesTableModel</t>
+          <t>HTMLList</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="B38" t="n">
         <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>StageRelocation</t>
+          <t>HtmlSelection</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="B39" t="n">
         <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TextUtilities</t>
+          <t>Interval</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="B40" t="n">
         <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Transform3D</t>
+          <t>MemberSet</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="B41" t="n">
         <v>1</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Translate2D</t>
+          <t>Pair</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B42" t="n">
         <v>1</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>UncertainValue</t>
+          <t>PrintUtilities</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="B43" t="n">
         <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>UncertainValue2</t>
+          <t>SpectrumPropertiesTableModel</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="B44" t="n">
         <v>1</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>UncertainValueMC</t>
+          <t>TextUtilities</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="B45" t="n">
         <v>1</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UtilException</t>
+          <t>Transform3D</t>
         </is>
       </c>
     </row>
@@ -14135,7 +15500,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AdaptiveRungeKutta</t>
+          <t>UtilException</t>
         </is>
       </c>
     </row>
@@ -14148,7 +15513,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AutoComplete</t>
+          <t>AdaptiveRungeKutta</t>
         </is>
       </c>
     </row>
@@ -14161,7 +15526,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ComboBoxCellEditor</t>
+          <t>AutoComplete</t>
         </is>
       </c>
     </row>
@@ -14174,7 +15539,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Constraint</t>
+          <t>ComboBoxCellEditor</t>
         </is>
       </c>
     </row>
@@ -14187,7 +15552,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CSVReader</t>
+          <t>HalfUpFormat</t>
         </is>
       </c>
     </row>
@@ -14200,7 +15565,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DescriptiveStatistics</t>
+          <t>ExponentFormat</t>
         </is>
       </c>
     </row>
@@ -14213,7 +15578,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EachRowEditor</t>
+          <t>FindRoot</t>
         </is>
       </c>
     </row>
@@ -14226,7 +15591,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ElementComboBoxModel</t>
+          <t>Math2</t>
         </is>
       </c>
     </row>
@@ -14239,7 +15604,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ElementTreePanel</t>
+          <t>UncertainValue2</t>
         </is>
       </c>
     </row>
@@ -14252,7 +15617,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ExponentFormat</t>
+          <t>Constraint</t>
         </is>
       </c>
     </row>
@@ -14265,7 +15630,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FindRoot</t>
+          <t>CSVReader</t>
         </is>
       </c>
     </row>
@@ -14278,7 +15643,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>HalfUpFormat</t>
+          <t>DescriptiveStatistics</t>
         </is>
       </c>
     </row>
@@ -14291,7 +15656,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Histogram</t>
+          <t>EachRowEditor</t>
         </is>
       </c>
     </row>
@@ -14304,7 +15669,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>HTMLFormat</t>
+          <t>ElementComboBoxModel</t>
         </is>
       </c>
     </row>
@@ -14317,7 +15682,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>HTMLList</t>
+          <t>ElementTreePanel</t>
         </is>
       </c>
     </row>
@@ -14330,7 +15695,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HtmlSelection</t>
+          <t>Histogram</t>
         </is>
       </c>
     </row>
@@ -14343,7 +15708,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Integrator</t>
+          <t>HTMLFormat</t>
         </is>
       </c>
     </row>
@@ -14356,7 +15721,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Interval</t>
+          <t>HTMLList</t>
         </is>
       </c>
     </row>
@@ -14369,7 +15734,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>LazyEvaluate</t>
+          <t>HtmlSelection</t>
         </is>
       </c>
     </row>
@@ -14382,7 +15747,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>LevenbergMarquardt2</t>
+          <t>Integrator</t>
         </is>
       </c>
     </row>
@@ -14395,7 +15760,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtConstrained</t>
+          <t>Interval</t>
         </is>
       </c>
     </row>
@@ -14408,7 +15773,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtParameterized</t>
+          <t>LazyEvaluate</t>
         </is>
       </c>
     </row>
@@ -14421,7 +15786,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>LinearLeastSquares</t>
+          <t>LevenbergMarquardt2</t>
         </is>
       </c>
     </row>
@@ -14434,7 +15799,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>LinearLeastSquaresMS</t>
+          <t>LevenbergMarquardtConstrained</t>
         </is>
       </c>
     </row>
@@ -14447,7 +15812,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LinearRegression</t>
+          <t>LevenbergMarquardtParameterized</t>
         </is>
       </c>
     </row>
@@ -14460,7 +15825,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Math2</t>
+          <t>LinearLeastSquares</t>
         </is>
       </c>
     </row>
@@ -14473,7 +15838,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MCIntegrator</t>
+          <t>LinearLeastSquaresMS</t>
         </is>
       </c>
     </row>
@@ -14486,7 +15851,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MCUncertaintyEngine</t>
+          <t>LinearRegression</t>
         </is>
       </c>
     </row>
@@ -14499,7 +15864,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MemberSet</t>
+          <t>MCIntegrator</t>
         </is>
       </c>
     </row>
@@ -14512,7 +15877,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MultiDHistogram</t>
+          <t>UncertainValueMC</t>
         </is>
       </c>
     </row>
@@ -14525,7 +15890,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pair</t>
+          <t>MCUncertaintyEngine</t>
         </is>
       </c>
     </row>
@@ -14538,7 +15903,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PoissonDeviate</t>
+          <t>MemberSet</t>
         </is>
       </c>
     </row>
@@ -14551,7 +15916,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PrintUtilities</t>
+          <t>MultiDHistogram</t>
         </is>
       </c>
     </row>
@@ -14564,7 +15929,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ProgressEvent</t>
+          <t>Pair</t>
         </is>
       </c>
     </row>
@@ -14577,7 +15942,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Simplex</t>
+          <t>PoissonDeviate</t>
         </is>
       </c>
     </row>
@@ -14590,7 +15955,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SpectrumPropertiesTableModel</t>
+          <t>PrintUtilities</t>
         </is>
       </c>
     </row>
@@ -14603,7 +15968,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>StageRelocation</t>
+          <t>ProgressEvent</t>
         </is>
       </c>
     </row>
@@ -14616,7 +15981,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TextUtilities</t>
+          <t>Simplex</t>
         </is>
       </c>
     </row>
@@ -14629,7 +15994,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Transform3D</t>
+          <t>SpectrumPropertiesTableModel</t>
         </is>
       </c>
     </row>
@@ -14642,7 +16007,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Translate2D</t>
+          <t>StageRelocation</t>
         </is>
       </c>
     </row>
@@ -14655,7 +16020,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>UncertainValue</t>
+          <t>TextUtilities</t>
         </is>
       </c>
     </row>
@@ -14668,7 +16033,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>UncertainValue2</t>
+          <t>Transform3D</t>
         </is>
       </c>
     </row>
@@ -14681,7 +16046,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>UncertainValueMC</t>
+          <t>Translate2D</t>
         </is>
       </c>
     </row>
@@ -14694,7 +16059,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>UtilException</t>
+          <t>UncertainValue</t>
         </is>
       </c>
     </row>
@@ -14768,7 +16133,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LinearLeastSquares</t>
+          <t>FindRoot</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -14793,14 +16158,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LevenbergMarquardt2</t>
+          <t>HalfUpFormat</t>
         </is>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -14818,20 +16183,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AdaptiveRungeKutta</t>
+          <t>Math2</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
@@ -14850,7 +16215,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -14868,20 +16233,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>UncertainValueMC</t>
+          <t>ExponentFormat</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G6" t="b">
         <v>0</v>
@@ -14897,16 +16262,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>0.3077</v>
       </c>
       <c r="G7" t="b">
         <v>0</v>
@@ -14918,20 +16283,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>UncertainValue</t>
+          <t>Constraint</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>0.3333</v>
       </c>
       <c r="G8" t="b">
         <v>0</v>
@@ -14943,20 +16308,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Translate2D</t>
+          <t>LevenbergMarquardt2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G9" t="b">
         <v>0</v>
@@ -14968,20 +16333,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Transform3D</t>
+          <t>Simplex</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>0.3333</v>
       </c>
       <c r="G10" t="b">
         <v>0</v>
@@ -14993,20 +16358,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>TextUtilities</t>
+          <t>DescriptiveStatistics</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G11" t="b">
         <v>0</v>
@@ -15018,20 +16383,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>StageRelocation</t>
+          <t>UncertainValueMC</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G12" t="b">
         <v>0</v>
@@ -15043,14 +16408,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SpectrumPropertiesTableModel</t>
+          <t>LazyEvaluate</t>
         </is>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -15068,20 +16433,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Simplex</t>
+          <t>LinearLeastSquares</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>0.6667</v>
       </c>
       <c r="G14" t="b">
         <v>0</v>
@@ -15093,20 +16458,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ProgressEvent</t>
+          <t>LevenbergMarquardtConstrained</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="G15" t="b">
         <v>0</v>
@@ -15118,20 +16483,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PrintUtilities</t>
+          <t>AdaptiveRungeKutta</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="G16" t="b">
         <v>0</v>
@@ -15143,20 +16508,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PoissonDeviate</t>
+          <t>UncertainValue</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="b">
         <v>0</v>
@@ -15168,20 +16533,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pair</t>
+          <t>Translate2D</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="b">
         <v>0</v>
@@ -15193,7 +16558,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MultiDHistogram</t>
+          <t>Transform3D</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -15218,7 +16583,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MemberSet</t>
+          <t>TextUtilities</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -15243,20 +16608,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MCUncertaintyEngine</t>
+          <t>StageRelocation</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="b">
         <v>0</v>
@@ -15268,7 +16633,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MCIntegrator</t>
+          <t>SpectrumPropertiesTableModel</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -15293,20 +16658,20 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Math2</t>
+          <t>ProgressEvent</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" t="b">
         <v>0</v>
@@ -15318,7 +16683,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>LinearRegression</t>
+          <t>PrintUtilities</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -15343,11 +16708,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LinearLeastSquaresMS</t>
+          <t>PoissonDeviate</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
@@ -15368,7 +16733,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtParameterized</t>
+          <t>Pair</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -15393,11 +16758,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LevenbergMarquardtConstrained</t>
+          <t>MultiDHistogram</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
@@ -15418,7 +16783,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>LazyEvaluate</t>
+          <t>MemberSet</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -15443,20 +16808,20 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Interval</t>
+          <t>MCUncertaintyEngine</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="b">
         <v>0</v>
@@ -15468,11 +16833,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Integrator</t>
+          <t>MCIntegrator</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
@@ -15493,20 +16858,20 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HtmlSelection</t>
+          <t>LinearRegression</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31" t="b">
         <v>0</v>
@@ -15518,20 +16883,20 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HTMLList</t>
+          <t>LinearLeastSquaresMS</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G32" t="b">
         <v>0</v>
@@ -15543,20 +16908,20 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HTMLFormat</t>
+          <t>LevenbergMarquardtParameterized</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33" t="b">
         <v>0</v>
@@ -15568,7 +16933,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Histogram</t>
+          <t>Interval</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -15593,20 +16958,20 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HalfUpFormat</t>
+          <t>Integrator</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G35" t="b">
         <v>0</v>
@@ -15618,7 +16983,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>FindRoot</t>
+          <t>HtmlSelection</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -15643,7 +17008,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ExponentFormat</t>
+          <t>HTMLList</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -15668,20 +17033,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ElementTreePanel</t>
+          <t>HTMLFormat</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G38" t="b">
         <v>0</v>
@@ -15693,7 +17058,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ElementComboBoxModel</t>
+          <t>Histogram</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -15718,7 +17083,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>EachRowEditor</t>
+          <t>ElementTreePanel</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -15743,7 +17108,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>DescriptiveStatistics</t>
+          <t>ElementComboBoxModel</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -15768,7 +17133,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CSVReader</t>
+          <t>EachRowEditor</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -15793,7 +17158,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Constraint</t>
+          <t>CSVReader</t>
         </is>
       </c>
       <c r="C43" t="n">

</xml_diff>